<commit_message>
Update tender documents with accurate dropdown values and audit results
Create a comprehensive audit report for tender documents, and update the Service-Resource-Model Excel file with precise dropdown values, ensuring alignment with TOGAF principles and the architectural blueprint.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: bd83b791-fe19-4f8c-8f08-c40cf927c2eb
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 80851d88-4415-415c-9797-c46c50695424
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/990d2e08-e877-47ab-86e4-4ab1ec4a5b18/bd83b791-fe19-4f8c-8f08-c40cf927c2eb/orRbN4m
</commit_message>
<xml_diff>
--- a/docs/gara-appalto/SERVICE-RESOURCE-MODEL-W3SUITE-v2.xlsx
+++ b/docs/gara-appalto/SERVICE-RESOURCE-MODEL-W3SUITE-v2.xlsx
@@ -5896,6 +5896,8 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="C102:C103"/>
+    <mergeCell ref="B256:D256"/>
     <mergeCell ref="B391:D391"/>
     <mergeCell ref="B378:D378"/>
     <mergeCell ref="B368:D368"/>
@@ -5912,8 +5914,6 @@
     <mergeCell ref="B98:B101"/>
     <mergeCell ref="C98:C101"/>
     <mergeCell ref="B102:B103"/>
-    <mergeCell ref="C102:C103"/>
-    <mergeCell ref="B256:D256"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -5924,46 +5924,46 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A4:AL17"/>
+  <dimension ref="A4:AL18"/>
   <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="20.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
-    <col min="7" max="7" width="20.83203125" customWidth="1"/>
-    <col min="8" max="8" width="20.83203125" customWidth="1"/>
-    <col min="9" max="9" width="20.83203125" customWidth="1"/>
-    <col min="10" max="10" width="20.83203125" customWidth="1"/>
-    <col min="11" max="11" width="20.83203125" customWidth="1"/>
-    <col min="12" max="12" width="20.83203125" customWidth="1"/>
-    <col min="13" max="13" width="20.83203125" customWidth="1"/>
-    <col min="14" max="14" width="20.83203125" customWidth="1"/>
-    <col min="15" max="15" width="20.83203125" customWidth="1"/>
-    <col min="16" max="16" width="20.83203125" customWidth="1"/>
-    <col min="17" max="17" width="20.83203125" customWidth="1"/>
-    <col min="18" max="18" width="20.83203125" customWidth="1"/>
-    <col min="19" max="19" width="20.83203125" customWidth="1"/>
-    <col min="20" max="20" width="20.83203125" customWidth="1"/>
-    <col min="21" max="21" width="20.83203125" customWidth="1"/>
-    <col min="22" max="22" width="20.83203125" customWidth="1"/>
-    <col min="23" max="23" width="20.83203125" customWidth="1"/>
-    <col min="24" max="24" width="20.83203125" customWidth="1"/>
-    <col min="25" max="25" width="20.83203125" customWidth="1"/>
-    <col min="26" max="26" width="20.83203125" customWidth="1"/>
-    <col min="27" max="27" width="20.83203125" customWidth="1"/>
-    <col min="28" max="28" width="20.83203125" customWidth="1"/>
-    <col min="29" max="29" width="20.83203125" customWidth="1"/>
-    <col min="30" max="30" width="20.83203125" customWidth="1"/>
-    <col min="31" max="31" width="20.83203125" customWidth="1"/>
-    <col min="32" max="32" width="20.83203125" customWidth="1"/>
-    <col min="33" max="33" width="20.83203125" customWidth="1"/>
-    <col min="34" max="34" width="20.83203125" customWidth="1"/>
-    <col min="35" max="35" width="20.83203125" customWidth="1"/>
-    <col min="36" max="36" width="20.83203125" customWidth="1"/>
-    <col min="37" max="37" width="20.83203125" customWidth="1"/>
-    <col min="38" max="38" width="20.83203125" customWidth="1"/>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="22.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" customWidth="1"/>
+    <col min="5" max="5" width="22.83203125" customWidth="1"/>
+    <col min="6" max="6" width="22.83203125" customWidth="1"/>
+    <col min="7" max="7" width="22.83203125" customWidth="1"/>
+    <col min="8" max="8" width="22.83203125" customWidth="1"/>
+    <col min="9" max="9" width="22.83203125" customWidth="1"/>
+    <col min="10" max="10" width="22.83203125" customWidth="1"/>
+    <col min="11" max="11" width="22.83203125" customWidth="1"/>
+    <col min="12" max="12" width="22.83203125" customWidth="1"/>
+    <col min="13" max="13" width="22.83203125" customWidth="1"/>
+    <col min="14" max="14" width="22.83203125" customWidth="1"/>
+    <col min="15" max="15" width="22.83203125" customWidth="1"/>
+    <col min="16" max="16" width="22.83203125" customWidth="1"/>
+    <col min="17" max="17" width="22.83203125" customWidth="1"/>
+    <col min="18" max="18" width="22.83203125" customWidth="1"/>
+    <col min="19" max="19" width="22.83203125" customWidth="1"/>
+    <col min="20" max="20" width="22.83203125" customWidth="1"/>
+    <col min="21" max="21" width="22.83203125" customWidth="1"/>
+    <col min="22" max="22" width="22.83203125" customWidth="1"/>
+    <col min="23" max="23" width="22.83203125" customWidth="1"/>
+    <col min="24" max="24" width="22.83203125" customWidth="1"/>
+    <col min="25" max="25" width="22.83203125" customWidth="1"/>
+    <col min="26" max="26" width="22.83203125" customWidth="1"/>
+    <col min="27" max="27" width="22.83203125" customWidth="1"/>
+    <col min="28" max="28" width="22.83203125" customWidth="1"/>
+    <col min="29" max="29" width="22.83203125" customWidth="1"/>
+    <col min="30" max="30" width="22.83203125" customWidth="1"/>
+    <col min="31" max="31" width="22.83203125" customWidth="1"/>
+    <col min="32" max="32" width="22.83203125" customWidth="1"/>
+    <col min="33" max="33" width="22.83203125" customWidth="1"/>
+    <col min="34" max="34" width="22.83203125" customWidth="1"/>
+    <col min="35" max="35" width="22.83203125" customWidth="1"/>
+    <col min="36" max="36" width="22.83203125" customWidth="1"/>
+    <col min="37" max="37" width="22.83203125" customWidth="1"/>
+    <col min="38" max="38" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="4">
@@ -6003,6 +6003,15 @@
       <c r="L4" t="str">
         <v/>
       </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v>Capacity  Model</v>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -6276,22 +6285,22 @@
         <v>Full IaaS</v>
       </c>
       <c r="H8" t="str">
-        <v>Seeweb S.r.l.</v>
+        <v>Seeweb S.r.l. (Cloud Italia)</v>
       </c>
       <c r="I8" t="str">
-        <v>Proxmox VE 8.x Virtualization Cluster</v>
+        <v>Proxmox VE 8.x Hypervisor Cluster</v>
       </c>
       <c r="J8" t="str">
         <v>3</v>
       </c>
       <c r="K8" t="str">
-        <v>Seeweb Italy (Rome DC)</v>
+        <v>Seeweb DC Italy (Rome/Milan)</v>
       </c>
       <c r="L8" t="str">
-        <v>Cloud-Multi-zone</v>
+        <v>Resources - SW configuration</v>
       </c>
       <c r="M8" t="str">
-        <v>Active-Active</v>
+        <v xml:space="preserve">Active </v>
       </c>
       <c r="N8" t="str">
         <v>Horizontal Scaling</v>
@@ -6312,16 +6321,16 @@
         <v>No</v>
       </c>
       <c r="T8" t="str">
-        <v>Proxmox cluster config</v>
+        <v>Proxmox cluster.conf</v>
       </c>
       <c r="U8" t="str">
-        <v>8.x</v>
+        <v>8.1.x</v>
       </c>
       <c r="V8" t="str">
-        <v>ISO/VM Template</v>
+        <v>ISO/VM Templates</v>
       </c>
       <c r="W8" t="str">
-        <v>Seeweb Infrastructure</v>
+        <v>Seeweb Internal</v>
       </c>
       <c r="X8" t="str">
         <v>DR</v>
@@ -6330,7 +6339,7 @@
         <v>Proxmox Backup Server</v>
       </c>
       <c r="Z8" t="str">
-        <v>Ceph</v>
+        <v>Ceph RGW</v>
       </c>
       <c r="AA8" t="str">
         <v>1 Day</v>
@@ -6339,7 +6348,7 @@
         <v>1 month</v>
       </c>
       <c r="AC8" t="str">
-        <v>5 min</v>
+        <v>1 min</v>
       </c>
       <c r="AD8" t="str">
         <v>1 week</v>
@@ -6360,13 +6369,13 @@
         <v>HW/SW vendor</v>
       </c>
       <c r="AJ8" t="str">
-        <v>Monitoring, Patching</v>
+        <v>Monitoring, Patching, Capacity</v>
       </c>
       <c r="AK8" t="str">
         <v>(on-premise) HW Buy &amp; Support</v>
       </c>
       <c r="AL8" t="str">
-        <v>Seeweb Cloud Italia</v>
+        <v>Seeweb Cloud Italia Contract</v>
       </c>
     </row>
     <row r="9">
@@ -6389,25 +6398,25 @@
         <v>Vendor Private</v>
       </c>
       <c r="G9" t="str">
-        <v>Full IaaS</v>
+        <v>HW Appliance</v>
       </c>
       <c r="H9" t="str">
         <v>Fortinet Inc.</v>
       </c>
       <c r="I9" t="str">
-        <v>FortiGate Next-Gen Firewall + WAF + IPS</v>
+        <v>FortiGate NGFW + WAF + IPS/IDS</v>
       </c>
       <c r="J9" t="str">
         <v>2</v>
       </c>
       <c r="K9" t="str">
-        <v>Seeweb Italy (Rome DC)</v>
+        <v>Seeweb DC Italy (Rome/Milan)</v>
       </c>
       <c r="L9" t="str">
-        <v>Cloud-Multi-zone</v>
+        <v>Resources - SW configuration</v>
       </c>
       <c r="M9" t="str">
-        <v>Active-StandBy</v>
+        <v xml:space="preserve">Active </v>
       </c>
       <c r="N9" t="str">
         <v>Fixed</v>
@@ -6431,13 +6440,13 @@
         <v>FortiOS config</v>
       </c>
       <c r="U9" t="str">
-        <v>7.x</v>
+        <v>7.4.x</v>
       </c>
       <c r="V9" t="str">
         <v>Firmware</v>
       </c>
       <c r="W9" t="str">
-        <v>Fortinet Support</v>
+        <v>Fortinet Support Portal</v>
       </c>
       <c r="X9" t="str">
         <v>DR</v>
@@ -6446,7 +6455,7 @@
         <v>Config Backup</v>
       </c>
       <c r="Z9" t="str">
-        <v>Ceph</v>
+        <v>Ceph RGW</v>
       </c>
       <c r="AA9" t="str">
         <v>1 Day</v>
@@ -6476,13 +6485,13 @@
         <v>HW/SW vendor</v>
       </c>
       <c r="AJ9" t="str">
-        <v>Security updates, Log review</v>
+        <v>Security Updates, Threat Monitoring</v>
       </c>
       <c r="AK9" t="str">
         <v>COTs SW License</v>
       </c>
       <c r="AL9" t="str">
-        <v>FortiCare subscription</v>
+        <v>FortiCare + FortiGuard</v>
       </c>
     </row>
     <row r="10">
@@ -6511,19 +6520,19 @@
         <v>W3Suite (Easy Digital Group)</v>
       </c>
       <c r="I10" t="str">
-        <v>Node.js 20 LTS + Express.js API Server</v>
+        <v>Node.js 20 LTS + Express.js REST API</v>
       </c>
       <c r="J10" t="str">
         <v>3</v>
       </c>
       <c r="K10" t="str">
-        <v>Seeweb Italy (Rome DC)</v>
+        <v>Seeweb DC Italy (Rome/Milan)</v>
       </c>
       <c r="L10" t="str">
-        <v>Cloud-Multi-zone</v>
+        <v>Resources - SW configuration</v>
       </c>
       <c r="M10" t="str">
-        <v>Active-Active</v>
+        <v xml:space="preserve">Active </v>
       </c>
       <c r="N10" t="str">
         <v>Horizontal Scaling</v>
@@ -6538,7 +6547,7 @@
         <v>Rolling</v>
       </c>
       <c r="R10" t="str">
-        <v>CI/CD Pipeline</v>
+        <v>Automated By App</v>
       </c>
       <c r="S10" t="str">
         <v>No</v>
@@ -6547,22 +6556,22 @@
         <v>package.json + env vars</v>
       </c>
       <c r="U10" t="str">
-        <v>Semantic versioning</v>
+        <v>SemVer</v>
       </c>
       <c r="V10" t="str">
-        <v>Docker image</v>
+        <v>Docker Image</v>
       </c>
       <c r="W10" t="str">
-        <v>Private Registry</v>
+        <v>Private Harbor Registry</v>
       </c>
       <c r="X10" t="str">
         <v>DR</v>
       </c>
       <c r="Y10" t="str">
-        <v>Container snapshot</v>
+        <v>Container Snapshot</v>
       </c>
       <c r="Z10" t="str">
-        <v>Ceph</v>
+        <v>Ceph RGW</v>
       </c>
       <c r="AA10" t="str">
         <v>1 Day</v>
@@ -6592,13 +6601,13 @@
         <v>SW Integrator</v>
       </c>
       <c r="AJ10" t="str">
-        <v>Release, Monitoring</v>
+        <v>CI/CD, Monitoring, Release</v>
       </c>
       <c r="AK10" t="str">
         <v>Subscription</v>
       </c>
       <c r="AL10" t="str">
-        <v>W3Suite SaaS license</v>
+        <v>W3Suite SaaS License</v>
       </c>
     </row>
     <row r="11">
@@ -6627,19 +6636,19 @@
         <v>F5 Networks (Nginx)</v>
       </c>
       <c r="I11" t="str">
-        <v>Nginx Reverse Proxy + Load Balancer + TLS</v>
+        <v>Nginx Reverse Proxy + TLS 1.3 Termination</v>
       </c>
       <c r="J11" t="str">
         <v>2</v>
       </c>
       <c r="K11" t="str">
-        <v>Seeweb Italy (Rome DC)</v>
+        <v>Seeweb DC Italy (Rome/Milan)</v>
       </c>
       <c r="L11" t="str">
-        <v>Cloud-Multi-zone</v>
+        <v>Resources - SW configuration</v>
       </c>
       <c r="M11" t="str">
-        <v>Active-Active</v>
+        <v xml:space="preserve">Active </v>
       </c>
       <c r="N11" t="str">
         <v>Horizontal Scaling</v>
@@ -6654,7 +6663,7 @@
         <v>Rolling</v>
       </c>
       <c r="R11" t="str">
-        <v>CI/CD Pipeline</v>
+        <v>Automated By App</v>
       </c>
       <c r="S11" t="str">
         <v>No</v>
@@ -6666,7 +6675,7 @@
         <v>1.24.x</v>
       </c>
       <c r="V11" t="str">
-        <v>Container image</v>
+        <v>Docker Image</v>
       </c>
       <c r="W11" t="str">
         <v>Docker Hub</v>
@@ -6675,10 +6684,10 @@
         <v>DR</v>
       </c>
       <c r="Y11" t="str">
-        <v>Config backup</v>
+        <v>Config Backup</v>
       </c>
       <c r="Z11" t="str">
-        <v>Ceph</v>
+        <v>Ceph RGW</v>
       </c>
       <c r="AA11" t="str">
         <v>1 Day</v>
@@ -6708,13 +6717,13 @@
         <v>SW Integrator</v>
       </c>
       <c r="AJ11" t="str">
-        <v>TLS renewal, Config updates</v>
+        <v>TLS Renewal, Config Updates</v>
       </c>
       <c r="AK11" t="str">
         <v>Subscription</v>
       </c>
       <c r="AL11" t="str">
-        <v>Open source + support</v>
+        <v>Open Source + Support</v>
       </c>
     </row>
     <row r="12">
@@ -6743,19 +6752,19 @@
         <v>Redis Ltd</v>
       </c>
       <c r="I12" t="str">
-        <v>Redis 7.x In-Memory Cache + Session Store</v>
+        <v>Redis 7.x In-Memory Cache + Session</v>
       </c>
       <c r="J12" t="str">
         <v>2</v>
       </c>
       <c r="K12" t="str">
-        <v>Seeweb Italy (Rome DC)</v>
+        <v>Seeweb DC Italy (Rome/Milan)</v>
       </c>
       <c r="L12" t="str">
-        <v>Cloud-Multi-zone</v>
+        <v>Resources - SW configuration</v>
       </c>
       <c r="M12" t="str">
-        <v>Master-Slave</v>
+        <v xml:space="preserve">Active </v>
       </c>
       <c r="N12" t="str">
         <v>Vertical Scaling</v>
@@ -6770,7 +6779,7 @@
         <v>Rolling</v>
       </c>
       <c r="R12" t="str">
-        <v>CI/CD Pipeline</v>
+        <v>Automated By App</v>
       </c>
       <c r="S12" t="str">
         <v>No</v>
@@ -6779,10 +6788,10 @@
         <v>redis.conf</v>
       </c>
       <c r="U12" t="str">
-        <v>7.x</v>
+        <v>7.2.x</v>
       </c>
       <c r="V12" t="str">
-        <v>Container image</v>
+        <v>Docker Image</v>
       </c>
       <c r="W12" t="str">
         <v>Docker Hub</v>
@@ -6791,10 +6800,10 @@
         <v>DR</v>
       </c>
       <c r="Y12" t="str">
-        <v>RDB snapshot + AOF</v>
+        <v>RDB + AOF</v>
       </c>
       <c r="Z12" t="str">
-        <v>Ceph</v>
+        <v>Ceph RGW</v>
       </c>
       <c r="AA12" t="str">
         <v>1 Day</v>
@@ -6803,7 +6812,7 @@
         <v>1 month</v>
       </c>
       <c r="AC12" t="str">
-        <v>5 min</v>
+        <v>1 min</v>
       </c>
       <c r="AD12" t="str">
         <v>1 week</v>
@@ -6824,13 +6833,13 @@
         <v>SW Integrator</v>
       </c>
       <c r="AJ12" t="str">
-        <v>Monitoring, Memory mgmt</v>
+        <v>Memory Monitoring, Cleanup</v>
       </c>
       <c r="AK12" t="str">
         <v>Subscription</v>
       </c>
       <c r="AL12" t="str">
-        <v>Open source</v>
+        <v>Open Source</v>
       </c>
     </row>
     <row r="13">
@@ -6856,7 +6865,7 @@
         <v>Mixed CaaS/PaaS</v>
       </c>
       <c r="H13" t="str">
-        <v>PostgreSQL Global Dev Group</v>
+        <v>PostgreSQL Global Development Group</v>
       </c>
       <c r="I13" t="str">
         <v>PostgreSQL 15 Primary + Streaming Replication</v>
@@ -6865,13 +6874,13 @@
         <v>2</v>
       </c>
       <c r="K13" t="str">
-        <v>Seeweb Italy (Rome DC)</v>
+        <v>Seeweb DC Italy (Rome/Milan)</v>
       </c>
       <c r="L13" t="str">
-        <v>Cloud-Multi-zone</v>
+        <v>Resources - SW configuration</v>
       </c>
       <c r="M13" t="str">
-        <v>Master-Slave</v>
+        <v xml:space="preserve">Active </v>
       </c>
       <c r="N13" t="str">
         <v>Vertical Scaling</v>
@@ -6880,7 +6889,7 @@
         <v>Manual By Operation</v>
       </c>
       <c r="P13" t="str">
-        <v>Yes (planned)</v>
+        <v>Yes (maintenance)</v>
       </c>
       <c r="Q13" t="str">
         <v>Rolling</v>
@@ -6889,7 +6898,7 @@
         <v>Manual By Operation</v>
       </c>
       <c r="S13" t="str">
-        <v>No</v>
+        <v>Planned</v>
       </c>
       <c r="T13" t="str">
         <v>postgresql.conf + pg_hba.conf</v>
@@ -6898,7 +6907,7 @@
         <v>15.x</v>
       </c>
       <c r="V13" t="str">
-        <v>Container image</v>
+        <v>Docker Image</v>
       </c>
       <c r="W13" t="str">
         <v>Docker Hub</v>
@@ -6907,10 +6916,10 @@
         <v>DR + Compliance</v>
       </c>
       <c r="Y13" t="str">
-        <v>pg_basebackup + WAL archiving</v>
+        <v>pg_basebackup + WAL Archive</v>
       </c>
       <c r="Z13" t="str">
-        <v>Ceph</v>
+        <v>Ceph RGW</v>
       </c>
       <c r="AA13" t="str">
         <v>1 Day</v>
@@ -6919,7 +6928,7 @@
         <v>1 month</v>
       </c>
       <c r="AC13" t="str">
-        <v>5 min</v>
+        <v>1 min</v>
       </c>
       <c r="AD13" t="str">
         <v>1 week</v>
@@ -6940,13 +6949,13 @@
         <v>SW Integrator</v>
       </c>
       <c r="AJ13" t="str">
-        <v>Backup, Tuning, Patching</v>
+        <v>Backup, Tuning, Patching, PITR</v>
       </c>
       <c r="AK13" t="str">
         <v>Subscription</v>
       </c>
       <c r="AL13" t="str">
-        <v>Open source + support</v>
+        <v>Open Source + Support</v>
       </c>
     </row>
     <row r="14">
@@ -6975,19 +6984,19 @@
         <v>Ceph Foundation (Red Hat)</v>
       </c>
       <c r="I14" t="str">
-        <v>Ceph Distributed Storage Cluster (RBD + CephFS)</v>
+        <v>Ceph Distributed Storage (RBD + CephFS + RGW)</v>
       </c>
       <c r="J14" t="str">
-        <v>3</v>
+        <v>3+</v>
       </c>
       <c r="K14" t="str">
-        <v>Seeweb Italy (Rome DC)</v>
+        <v>Seeweb DC Italy (Rome/Milan)</v>
       </c>
       <c r="L14" t="str">
-        <v>Cloud-Multi-zone</v>
+        <v>Resources - SW configuration</v>
       </c>
       <c r="M14" t="str">
-        <v>Active-Active</v>
+        <v xml:space="preserve">Active </v>
       </c>
       <c r="N14" t="str">
         <v>Horizontal Scaling</v>
@@ -7017,16 +7026,16 @@
         <v>Packages</v>
       </c>
       <c r="W14" t="str">
-        <v>Ceph repo</v>
+        <v>Ceph Official Repo</v>
       </c>
       <c r="X14" t="str">
         <v>DR</v>
       </c>
       <c r="Y14" t="str">
-        <v>Ceph snapshots + RGW replication</v>
+        <v>Ceph Snapshots + RGW Replication</v>
       </c>
       <c r="Z14" t="str">
-        <v>Ceph (self)</v>
+        <v>Ceph (self-replicating)</v>
       </c>
       <c r="AA14" t="str">
         <v>1 Day</v>
@@ -7035,7 +7044,7 @@
         <v>1 month</v>
       </c>
       <c r="AC14" t="str">
-        <v>5 min</v>
+        <v>1 min</v>
       </c>
       <c r="AD14" t="str">
         <v>1 week</v>
@@ -7056,7 +7065,7 @@
         <v>HW/SW vendor</v>
       </c>
       <c r="AJ14" t="str">
-        <v>Capacity, Health monitoring</v>
+        <v>Capacity, Health, OSD Management</v>
       </c>
       <c r="AK14" t="str">
         <v>(on-premise) HW Buy &amp; Support</v>
@@ -7097,13 +7106,13 @@
         <v>N/A (SaaS)</v>
       </c>
       <c r="K15" t="str">
-        <v>OpenAI Cloud (EU endpoint)</v>
+        <v>OpenAI Cloud (EU Endpoint)</v>
       </c>
       <c r="L15" t="str">
-        <v xml:space="preserve">Cloud-Multi-region </v>
+        <v xml:space="preserve">Internal SaaS/Cloud provider -configuration  </v>
       </c>
       <c r="M15" t="str">
-        <v>Active-Active</v>
+        <v xml:space="preserve">Active </v>
       </c>
       <c r="N15" t="str">
         <v>On Demand</v>
@@ -7124,7 +7133,7 @@
         <v>No</v>
       </c>
       <c r="T15" t="str">
-        <v>API Key + Org settings</v>
+        <v>API Key + Organization</v>
       </c>
       <c r="U15" t="str">
         <v>API v1</v>
@@ -7172,7 +7181,7 @@
         <v>SaaS Provider</v>
       </c>
       <c r="AJ15" t="str">
-        <v>API monitoring</v>
+        <v>API Usage Monitoring</v>
       </c>
       <c r="AK15" t="str">
         <v>Subscription</v>
@@ -7213,13 +7222,13 @@
         <v>2</v>
       </c>
       <c r="K16" t="str">
-        <v>Seeweb Italy (Rome DC)</v>
+        <v>Seeweb DC Italy (Rome/Milan)</v>
       </c>
       <c r="L16" t="str">
-        <v>Cloud-Multi-zone</v>
+        <v>Resources - SW configuration</v>
       </c>
       <c r="M16" t="str">
-        <v>Active-Active</v>
+        <v xml:space="preserve">Active </v>
       </c>
       <c r="N16" t="str">
         <v>Horizontal Scaling</v>
@@ -7234,31 +7243,31 @@
         <v>Rolling</v>
       </c>
       <c r="R16" t="str">
-        <v>CI/CD Pipeline</v>
+        <v>Automated By App</v>
       </c>
       <c r="S16" t="str">
         <v>No</v>
       </c>
       <c r="T16" t="str">
-        <v>MCP config + action_definitions</v>
+        <v>action_definitions + MCP config</v>
       </c>
       <c r="U16" t="str">
-        <v>Semantic versioning</v>
+        <v>SemVer</v>
       </c>
       <c r="V16" t="str">
-        <v>Docker image</v>
+        <v>Docker Image</v>
       </c>
       <c r="W16" t="str">
-        <v>Private Registry</v>
+        <v>Private Harbor Registry</v>
       </c>
       <c r="X16" t="str">
         <v>DR</v>
       </c>
       <c r="Y16" t="str">
-        <v>Config backup</v>
+        <v>Config + DB Backup</v>
       </c>
       <c r="Z16" t="str">
-        <v>Ceph</v>
+        <v>Ceph RGW</v>
       </c>
       <c r="AA16" t="str">
         <v>1 Day</v>
@@ -7288,13 +7297,13 @@
         <v>SW Integrator</v>
       </c>
       <c r="AJ16" t="str">
-        <v>Monitoring, Routing rules</v>
+        <v>Routing Rules, Provider Mgmt</v>
       </c>
       <c r="AK16" t="str">
         <v>Subscription</v>
       </c>
       <c r="AL16" t="str">
-        <v>W3Suite SaaS license</v>
+        <v>W3Suite SaaS License</v>
       </c>
     </row>
     <row r="17">
@@ -7329,13 +7338,13 @@
         <v>3</v>
       </c>
       <c r="K17" t="str">
-        <v>Seeweb Italy (Rome DC)</v>
+        <v>Seeweb DC Italy (Rome/Milan)</v>
       </c>
       <c r="L17" t="str">
-        <v>Cloud-Multi-zone</v>
+        <v>Resources - SW configuration</v>
       </c>
       <c r="M17" t="str">
-        <v>Active-Active</v>
+        <v xml:space="preserve">Active </v>
       </c>
       <c r="N17" t="str">
         <v>Horizontal Scaling</v>
@@ -7350,7 +7359,7 @@
         <v>Rolling</v>
       </c>
       <c r="R17" t="str">
-        <v>CI/CD Pipeline</v>
+        <v>Automated By App</v>
       </c>
       <c r="S17" t="str">
         <v>No</v>
@@ -7359,22 +7368,22 @@
         <v>Auth config + RBAC policies</v>
       </c>
       <c r="U17" t="str">
-        <v>Semantic versioning</v>
+        <v>SemVer</v>
       </c>
       <c r="V17" t="str">
-        <v>Docker image</v>
+        <v>Docker Image</v>
       </c>
       <c r="W17" t="str">
-        <v>Private Registry</v>
+        <v>Private Harbor Registry</v>
       </c>
       <c r="X17" t="str">
         <v>Compliance</v>
       </c>
       <c r="Y17" t="str">
-        <v>DB backup (auth data)</v>
+        <v>DB Backup (auth tables)</v>
       </c>
       <c r="Z17" t="str">
-        <v>Ceph</v>
+        <v>Ceph RGW</v>
       </c>
       <c r="AA17" t="str">
         <v>1 Day</v>
@@ -7383,7 +7392,7 @@
         <v>1 month</v>
       </c>
       <c r="AC17" t="str">
-        <v>5 min</v>
+        <v>1 min</v>
       </c>
       <c r="AD17" t="str">
         <v>1 week</v>
@@ -7404,18 +7413,134 @@
         <v>SW Integrator</v>
       </c>
       <c r="AJ17" t="str">
-        <v>Security audits, Key rotation</v>
+        <v>Key Rotation, Audit, MFA Config</v>
       </c>
       <c r="AK17" t="str">
         <v>Subscription</v>
       </c>
       <c r="AL17" t="str">
-        <v>W3Suite SaaS license</v>
+        <v>W3Suite SaaS License</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>PROD</v>
+      </c>
+      <c r="B18" t="str">
+        <v>99,5%</v>
+      </c>
+      <c r="C18" t="str">
+        <v>HA-</v>
+      </c>
+      <c r="D18" t="str">
+        <v>OBSERVABILITY</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Not W3 Private datacenter</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Vendor Private</v>
+      </c>
+      <c r="G18" t="str">
+        <v>Mixed CaaS/PaaS</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Grafana Labs</v>
+      </c>
+      <c r="I18" t="str">
+        <v>Grafana + Prometheus + Loki Stack</v>
+      </c>
+      <c r="J18" t="str">
+        <v>2</v>
+      </c>
+      <c r="K18" t="str">
+        <v>Seeweb DC Italy (Rome/Milan)</v>
+      </c>
+      <c r="L18" t="str">
+        <v>Resources - SW configuration</v>
+      </c>
+      <c r="M18" t="str">
+        <v xml:space="preserve">Active </v>
+      </c>
+      <c r="N18" t="str">
+        <v>Horizontal Scaling</v>
+      </c>
+      <c r="O18" t="str">
+        <v>Manual By Operation</v>
+      </c>
+      <c r="P18" t="str">
+        <v>No</v>
+      </c>
+      <c r="Q18" t="str">
+        <v>Rolling</v>
+      </c>
+      <c r="R18" t="str">
+        <v>Automated By App</v>
+      </c>
+      <c r="S18" t="str">
+        <v>No</v>
+      </c>
+      <c r="T18" t="str">
+        <v>prometheus.yml + grafana.ini</v>
+      </c>
+      <c r="U18" t="str">
+        <v>10.x</v>
+      </c>
+      <c r="V18" t="str">
+        <v>Docker Image</v>
+      </c>
+      <c r="W18" t="str">
+        <v>Docker Hub</v>
+      </c>
+      <c r="X18" t="str">
+        <v>DR</v>
+      </c>
+      <c r="Y18" t="str">
+        <v>Config + Dashboard Export</v>
+      </c>
+      <c r="Z18" t="str">
+        <v>Ceph RGW</v>
+      </c>
+      <c r="AA18" t="str">
+        <v>1 Day</v>
+      </c>
+      <c r="AB18" t="str">
+        <v>1 month</v>
+      </c>
+      <c r="AC18" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="AD18" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="AE18" t="str">
+        <v xml:space="preserve">Local Resilent </v>
+      </c>
+      <c r="AF18" t="str">
+        <v>Manual By Operation</v>
+      </c>
+      <c r="AG18" t="str">
+        <v>Hour (1-5)</v>
+      </c>
+      <c r="AH18" t="str">
+        <v>Hour (1-5)</v>
+      </c>
+      <c r="AI18" t="str">
+        <v>SW Integrator</v>
+      </c>
+      <c r="AJ18" t="str">
+        <v>Dashboard Creation, Alert Rules</v>
+      </c>
+      <c r="AK18" t="str">
+        <v>Subscription</v>
+      </c>
+      <c r="AL18" t="str">
+        <v>Open Source</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A4:AL17"/>
+    <ignoredError numberStoredAsText="1" sqref="A4:AL18"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>